<commit_message>
update final for today
</commit_message>
<xml_diff>
--- a/exports/FR_Budget_Status.xlsx
+++ b/exports/FR_Budget_Status.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Open Line FR Report - As On 05." sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Open Line FR Fund Wise - As On " sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="GSU FR Report - As On 05.09.202" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="GSU FR Fund Wise - As On 05.09." sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Line FR Report - As On 05." sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Line FR Fund Wise - As On " sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GSU FR Report - As On 05.09.202" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GSU FR Fund Wise - As On 05.09." sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -565,20 +565,71 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>160,903
-Cr. 16.09</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>160,903</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>16.09 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>77,992
-Cr. 7.80</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>77,992</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>7.80 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>-82,911
-Cr. -8.29</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-82,911</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-8.29 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -600,20 +651,71 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>32,227
-Cr. 3.22</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>32,227</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>3.22 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>11,801
-Cr. 1.18</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>11,801</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>1.18 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>-20,426
-Cr. -2.04</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-20,426</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-2.04 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -635,20 +737,71 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>120,318
-Cr. 12.03</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>120,318</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>12.03 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>57,289
-Cr. 5.73</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>57,289</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>5.73 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>-63,029
-Cr. -6.30</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-63,029</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-6.30 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -670,20 +823,71 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>507,420
-Cr. 50.74</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>507,420</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>50.74 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>363,937
-Cr. 36.39</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>363,937</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>36.39 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>-143,483
-Cr. -14.35</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-143,483</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-14.35 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -705,20 +909,71 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2,962,795
-Cr. 296.28</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>2,962,795</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>296.28 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>3,692,699
-Cr. 369.27</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>3,692,699</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>369.27 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>729,904
-Cr. 72.99</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>729,904</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>72.99 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -740,20 +995,71 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>132,267
-Cr. 13.23</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>132,267</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>13.23 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>151,197
-Cr. 15.12</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>151,197</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>15.12 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>18,930
-Cr. 1.89</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>18,930</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>1.89 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -775,20 +1081,71 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>522,843
-Cr. 52.28</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>522,843</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>52.28 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>123,038
-Cr. 12.30</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>123,038</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>12.30 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>-399,805
-Cr. -39.98</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-399,805</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-39.98 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -810,20 +1167,71 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>307,843
-Cr. 30.78</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>307,843</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>30.78 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>94,924
-Cr. 9.49</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>94,924</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>9.49 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>-212,919
-Cr. -21.29</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-212,919</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-21.29 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -845,20 +1253,71 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -880,20 +1339,71 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>13,194
-Cr. 1.32</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>13,194</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>1.32 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>24,273
-Cr. 2.43</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>24,273</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>2.43 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>11,079
-Cr. 1.11</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>11,079</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>1.11 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -915,20 +1425,71 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>53,702
-Cr. 5.37</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>53,702</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>5.37 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>5,129
-Cr. 0.51</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>5,129</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.51 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>-48,573
-Cr. -4.86</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-48,573</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-4.86 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -950,20 +1511,71 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>97,500
-Cr. 9.75</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>97,500</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>9.75 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>59,852
-Cr. 5.99</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>59,852</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>5.99 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>-37,648
-Cr. -3.76</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-37,648</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-3.76 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -985,20 +1597,71 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>310,912
-Cr. 31.09</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>310,912</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>31.09 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>131,048
-Cr. 13.10</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>131,048</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>13.10 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>-179,864
-Cr. -17.99</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-179,864</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-17.99 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1020,20 +1683,71 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1055,20 +1769,71 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>315,733
-Cr. 31.57</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>315,733</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>31.57 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>103,375
-Cr. 10.34</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>103,375</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>10.34 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>-212,358
-Cr. -21.24</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-212,358</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-21.24 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1086,20 +1851,71 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>64,034
-Cr. 6.40</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>64,034</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>6.40 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>-64,034
-Cr. -6.40</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-64,034</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-6.40 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -1121,20 +1937,71 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>6,010
-Cr. 0.60</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>6,010</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.60 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>-6,010
-Cr. -0.60</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-6,010</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-0.60 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1152,20 +2019,71 @@
       <c r="B22" s="5" t="inlineStr"/>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>5,607,701
-Cr. 560.77</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>5,607,701</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>560.77 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>4,896,554
-Cr. 489.66</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>4,896,554</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>489.66 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>-711,147
-Cr. -71.11</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-711,147</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-71.11 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -1269,20 +2187,71 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>1,018,353
-Cr. 101.84</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>1,018,353</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>101.84 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>408,842
-Cr. 40.88</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>408,842</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>40.88 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>609,511
-Cr. 60.95</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>609,511</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>60.95 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1304,20 +2273,71 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>40,232
-Cr. 4.02</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>40,232</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>4.02 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>15,491
-Cr. 1.55</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>15,491</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>1.55 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>24,741
-Cr. 2.47</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>24,741</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>2.47 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -1339,20 +2359,71 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>130,592
-Cr. 13.06</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>130,592</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>13.06 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>18,459
-Cr. 1.85</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>18,459</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>1.85 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>112,133
-Cr. 11.21</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>112,133</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>11.21 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1374,20 +2445,71 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1409,20 +2531,71 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>3,117,515
-Cr. 311.75</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>3,117,515</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>311.75 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>3,746,106
-Cr. 374.61</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>3,746,106</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>374.61 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>-628,591
-Cr. -62.86</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-628,591</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-62.86 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1444,20 +2617,71 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -1479,20 +2703,71 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>1,301,009
-Cr. 130.10</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>1,301,009</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>130.10 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>707,656
-Cr. 70.77</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>707,656</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>70.77 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>593,353
-Cr. 59.34</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>593,353</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>59.34 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1606,20 +2881,71 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -1641,20 +2967,71 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -1676,20 +3053,71 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1711,20 +3139,71 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>1
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>1</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>127
-Cr. 0.01</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>127</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.01 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>126
-Cr. 0.01</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>126</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.01 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -1746,20 +3225,71 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1781,20 +3311,71 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -1816,20 +3397,71 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1851,20 +3483,71 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -1886,20 +3569,71 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1921,20 +3655,71 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>1
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>1</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>-1
-Cr. -0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-1</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1956,20 +3741,71 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>5,001
-Cr. 0.50</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>5,001</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.50 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>2,048
-Cr. 0.20</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>2,048</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.20 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>-2,953
-Cr. -0.30</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-2,953</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-0.30 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1991,20 +3827,71 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -2026,20 +3913,71 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>446,600
-Cr. 44.66</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>446,600</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>44.66 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>317,088
-Cr. 31.71</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>317,088</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>31.71 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>-129,512
-Cr. -12.95</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-129,512</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-12.95 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -2061,20 +3999,71 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -2096,20 +4085,71 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -2127,20 +4167,71 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -2162,20 +4253,71 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -2193,20 +4335,71 @@
       <c r="B22" s="5" t="inlineStr"/>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>451,603
-Cr. 45.16</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>451,603</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>45.16 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>319,263
-Cr. 31.93</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>319,263</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>31.93 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>-132,340
-Cr. -13.23</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-132,340</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-13.23 Cr</t>
+          </r>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -2310,20 +4503,71 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>451,601
-Cr. 45.16</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>451,601</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>45.16 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>319,136
-Cr. 31.91</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>319,136</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>31.91 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>132,465
-Cr. 13.25</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>132,465</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>13.25 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -2345,20 +4589,71 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>1
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>1</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>1
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>1</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -2380,20 +4675,71 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -2415,20 +4761,71 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -2450,20 +4847,71 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -2485,20 +4933,71 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>0
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>0</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -2520,20 +5019,71 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>1
-Cr. 0.00</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>1</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.00 Cr</t>
+          </r>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>127
-Cr. 0.01</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>127</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>0.01 Cr</t>
+          </r>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>-126
-Cr. -0.01</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>-126</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <color rgb="FF006F78"/>
+              <sz val="9"/>
+            </rPr>
+            <t>-0.01 Cr</t>
+          </r>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">

</xml_diff>